<commit_message>
tracker: log both waiter order-placement crashes (rows 73, 78)
Row 73: the v3.6 fix - .data('select2') guarded at 29 sites, corrected scope
(ALL order types, not Club-specific).
Row 78: the v3.7 follow-up - .select2('data') at three earlier sites, plus the
view/JS flag mismatch ($is_waiter_user vs waiter_app_status) that made my v3.6
test fixture validate the wrong shape and miss it.

Also logs the icon-filename spacing item, the single_item markup regression, the
mobile hover-only category rail, and the dark theme rebuild.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/doc/Rexlio_POS_Task_Tracker.xlsx
+++ b/doc/Rexlio_POS_Task_Tracker.xlsx
@@ -611,7 +611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E72"/>
+  <dimension ref="A1:E78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2562,6 +2562,168 @@
       <c r="E72" s="25" t="inlineStr">
         <is>
           <t>Tested the real Rockbell_Lounge_Menu.xlsx (174 rows) end to end through the uploader on the scratch clone. READABILITY IS FINE - no Excel re-save is required. Although created by openpyxl the file was last saved by LibreOffice 24.2.7.2, and PHPExcel parses it cleanly (174 rows, all values). That matters because PHPExcel CANNOT read a pure openpyxl-written file at all - it warns in Excel2007.php:457 and returns an empty sheet - though it fails safe, rejecting rather than importing garbage. STRUCTURE IS THE BLOCKER. The file is Category | Sub Category | Item | Variant | Regular | Takeaway | Delivery | VIP | Club with headers on row 1; the template is Name | Code | Category | Regular | Takeaway | Delivery | Tax Name | Tax % | Description | Veg | Beverage | Image | Loyalty | Alt Name | VIP | Club with headers on row 3 and data from row 4. Upload was rejected with column D/J/K errors and imported nothing. Also unmapped: there is no Code column (Code is required); Sub Category has nowhere to go because food menu categories are FLAT (no parent_id on tbl_food_menu_categories); and Variant implies variations, which the vendor template explicitly says to exclude from bulk upload. A transform step is needed, plus decisions on code generation, sub-category handling and variants.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Incident</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>[CRITICAL - FIXED] Waiters could not place orders on ANY order type</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Done - fixed and verified</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>SEVERITY CORRECTED BY USER: this affects EVERY order type and EVERY waiter. It was first seen on a Club-locked counter, and my initial report wrongly scoped it as Club/counter-lock specific - the lock was incidental to where testing happened, not the trigger. Reproduced identically on local AND the fresh live Rockbell deployment. SYMPTOM: waiter selects items normally, clicks Place Order, nothing happens - no request, no message, no visible error. CAUSE: waiter self-attribution renders #select_waiter as a fixed hidden INPUT instead of &lt;select class=select2&gt;, but the order handlers called $('#select_waiter').data('select2').open()/.close() unguarded. For a waiter that resolves to undefined, so it threw TypeError INSIDE the .place_order_operation click handler, killing it before the request was built. jQuery does not surface it, so the button looked dead. Role-specific: Admin/Cashier/Manager get a real select2, so the same line correctly opens the prompt. SCOPE - every branch of the order-type chain carries the same unguarded calls: delivery_button (customer_id=='' | customer_id=='1' | address==''), dine_in|vip|club (waiter_id=='' | customer_id==''), take_away (waiter_id=='' | customer_id==''). Delivery was worst: it also refuses walk-in (customer_id=='1'), so a waiter on the default customer crashed there even WITH a customer selected. FIX: all 29 op1/op2 .open()/.close() calls made null-safe - identical behaviour where the dropdown exists, nudge skipped where it does not. 28 in the order paths (.place_order_operation, #direct_invoice); the 29th (.same_or_diff_state_modal) is the same crash class and was guarded too. An assertion caught that 29th site, which I would otherwise have missed. VERIFIED (measured, not inferred) - waiter session, register open, item in cart. BEFORE (pre-fix script restored, order type forced at attribute level because the counter lock stops a waiter switching it in the UI): Regular/Outlet/Delivery/VIP/Club with no customer -&gt; TypeError, 0 requests; Delivery+walk-in -&gt; TypeError, 0 requests. AFTER, each on a FRESH page load: Regular, Outlet, VIP, Club and Delivery+real customer all -&gt; no crash, POST Sale/add_kitchen_sale_by_ajax fires; Delivery+walk-in -&gt; no crash, refuses cleanly (correct - walk-in is not a valid delivery customer). METHOD NOTE: my first matrix was INVALID and I caught it before reporting - selected_ok was false on 4 of 5 rows, meaning the order type never actually switched and all five trials re-ran the same branch; and a later single-page run was contaminated by state left by the previous trial, so the final matrix uses one fresh page load per order type. RULED OUT: register gate (waiter loaded the POS with registers open at the outlet - and it fails loudly, redirecting away from the POS entirely), zero-stock block (only in add-to-cart paths, and it fails open), server guards (they return an invoice_msg the app displays, so they cannot produce silence). DEPLOY: commit a968d3e1 - pos_script_v7.3.js plus main_screen.php carrying the ?v=3.5-&gt;3.6 cache bust IN THE SAME COMMIT; without that bump tills keep the broken cached script.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Category icon filenames contain spaces (Beer Mug.png, etc.)</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Logged - not scheduled</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Flagged during the UI redesign, deliberately not fixed. Several icon assets are named with spaces. They work because the browser percent-encodes the space, but such names break naive URL building, some cache/CDN layers, and unquoted shell handling. Rename to hyphenated lowercase AND update references in one change - renaming the files alone breaks the pages pointing at them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Redesign</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>[Regression - FOUND AND FIXED] POS category grids lost their tile markup</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Done - fixed and verified</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Introduced by my own thumbnail patch, caught only when the redesign was click-tested through a real order flow. pos_thumb_fix.py sliced out a region ending at '$menu_to_show .= $ir_thumb;' then tried to re-emit the &lt;img&gt; with a .replace() on that same string; the slice had consumed it, so the replace matched nothing and SILENTLY no-oped. Lost: the &lt;div class=single_item&gt; wrapper (data-price*, id=item_N), the &lt;img&gt;, and the $food_menu_tooltip/$item_name_c block, leaving an orphaned &lt;/div&gt;. Live effect: the default grid still worked (JS-built from window.items) but clicking ANY category rendered bare name/price text, no image, NOT clickable. Same silent-no-op mode as the userHome.php menu-list break: a .replace() whose match may already be consumed now requires an assertion. After fix: 197 tiles, 197 images, 33 holders, 0 notices.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Next</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>[Base-product] Mobile category rail opens on CSS :hover only</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Logged - not scheduled</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Found while click-testing the redesign at 375x812. The mobile category surface (.all__menus, toggled by .show_all_menu) reveals categories via '.it_has_children:hover .sub_menu' (style2.css:2523). Hover does not exist on touch, so on a waiter tablet those categories may be unreachable. Vendor behaviour, NOT caused by the redesign, and NOT verified on real touch hardware - flagged only. Desktop rail unaffected (33/33 clickable, light and dark).</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Redesign</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Dark theme rebuilt to match the supplied mockup (POS + dashboard)</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Done - verified</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>User feedback on the first dark pass: category buttons too rounded, too much white. Root cause of the white: the first pass themed the CONTENT of the sale screen but not the PANELS - style2.css paints .main_left/.main_middle/.main_right/.main_center/.holder/.top_header_part a hardcoded #fff. Added theme sections 15-21. Category radius 9px-&gt;4px. All painted FROM TOKENS so light is unchanged (--rx-surface IS #fff in light) - re-measured light after the change and every surface matched. Separators use inset box-shadow, never border, so no element gains box size. RESULTS: POS on-screen light surfaces 23-&gt;2 (both intentional brand greens); low-contrast text 9-&gt;4 (the 4 remaining are white-on-brand pills identical in LIGHT too, i.e. pre-existing). Dashboard: 11 white KPI slabs -&gt; 0 light surfaces, 0 low-contrast, charts intact. CHART FIX: the dashboard loads TWO Chart.js builds (v3 then v2, v2 overwriting window.Chart), so Chart.getChart() was undefined and my retint was a silent no-op; the vendor also sets borderColor '#00000000' and defines no scales at all. Chart now hands its instance to the theme layer. Hit-testing re-run after the CSS: 19/19 categories, 12/12 tiles, 2/2 order buttons, 6/6 operation buttons, IDENTICAL with the theme on and off.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Incident</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>[CRITICAL - FIXED] Second waiter crash: .select2('data') on hidden waiter field</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Done - fixed and verified</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>FOLLOW-UP to row 73. The v3.6 fix was real but INCOMPLETE, and my verification of it was flawed. v3.6 guarded .data('select2') results (op1/op2, 29 sites, all still correct). This is a DIFFERENT select2 API on the same element - .select2('data') - at three sites sitting EARLIER in the same handler, so the click died at line 8479 and never reached the guarded code at 8530+. Error: "Uncaught TypeError: Cannot read properties of undefined (reading 'data')", preceded by select2's own warning "The select2('data') method was called on an element that is not using Select2". No order request ever reached the network. WHY MY v3.6 TESTING MISSED IT - the view and the JS branch on two DIFFERENT flags: the view renders #select_waiter as a hidden input when $is_waiter_user (isWaiterUser() = session designation=='Waiter' OR is_waiter=='Yes'), while the JS called .select2('data') when waiter_app_status!='Yes', and main_screen.php:5 sets $waiter_app_status = session is_waiter. So a waiter with designation 'Waiter' but is_waiter NOT 'Yes' gets the hidden input AND takes the select2 path. My test session set is_waiter='Yes', which took the safe else branch and hid the bug; production waiters have is_waiter='No'. THE FLAG MISMATCH IS THE REAL DEFECT - the crash is only its symptom. LESSON: my test fixture was built to satisfy the feature's own happy path rather than to match production, so it validated the wrong shape. FIX: new irWaiterName() helper tests the ELEMENT, not a flag - uses .select2('data') only when #select_waiter really is a select carrying a select2 instance, else reads #select_waiter_name (which the view always emits beside the hidden input). Applied at all three sites: 8479 (.place_order_operation, was guarded by the WRONG flag), 9023 (#direct_invoice, completely unguarded), 9711 (split payment, completely unguarded). The latter two had no flag check at all and so crashed for ANY waiter. VERIFIED on the production session shape (designation=Waiter, is_waiter=No, hidden INPUT, waiter_app_status renders 'No'), user's exact steps - Cup Yogurt, total 3000.00, Place Order: v3.6 -&gt; TypeError reading 'data', 0 order requests; v3.7 -&gt; no error, POST Sale/add_kitchen_sale_by_ajax fires. Admin regression same build: no crash, waiter dropdown still opens (select2-container--open=2), so behaviour unchanged where a real select2 exists. DEPLOY: commit 48936b4e - pos_script_v7.3.js + main_screen.php carrying ?v=3.6-&gt;3.7 in the SAME commit.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: log the register force-close and category rail work in the tracker
Two rows appended, 78 -> 80. Row 79 covers the Admin register force-close
feature (commits 84a0f165, ef75e0ec), including the verification lesson from
it - a DOM proof run against the scratch database is not evidence about
production, and "verified" needs to name which database it was verified
against. Row 80 covers the category rail redesign (commit f76a2106).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/doc/Rexlio_POS_Task_Tracker.xlsx
+++ b/doc/Rexlio_POS_Task_Tracker.xlsx
@@ -611,7 +611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E78"/>
+  <dimension ref="A1:E80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2724,6 +2724,60 @@
       <c r="E78" t="inlineStr">
         <is>
           <t>FOLLOW-UP to row 73. The v3.6 fix was real but INCOMPLETE, and my verification of it was flawed. v3.6 guarded .data('select2') results (op1/op2, 29 sites, all still correct). This is a DIFFERENT select2 API on the same element - .select2('data') - at three sites sitting EARLIER in the same handler, so the click died at line 8479 and never reached the guarded code at 8530+. Error: "Uncaught TypeError: Cannot read properties of undefined (reading 'data')", preceded by select2's own warning "The select2('data') method was called on an element that is not using Select2". No order request ever reached the network. WHY MY v3.6 TESTING MISSED IT - the view and the JS branch on two DIFFERENT flags: the view renders #select_waiter as a hidden input when $is_waiter_user (isWaiterUser() = session designation=='Waiter' OR is_waiter=='Yes'), while the JS called .select2('data') when waiter_app_status!='Yes', and main_screen.php:5 sets $waiter_app_status = session is_waiter. So a waiter with designation 'Waiter' but is_waiter NOT 'Yes' gets the hidden input AND takes the select2 path. My test session set is_waiter='Yes', which took the safe else branch and hid the bug; production waiters have is_waiter='No'. THE FLAG MISMATCH IS THE REAL DEFECT - the crash is only its symptom. LESSON: my test fixture was built to satisfy the feature's own happy path rather than to match production, so it validated the wrong shape. FIX: new irWaiterName() helper tests the ELEMENT, not a flag - uses .select2('data') only when #select_waiter really is a select carrying a select2 instance, else reads #select_waiter_name (which the view always emits beside the hidden input). Applied at all three sites: 8479 (.place_order_operation, was guarded by the WRONG flag), 9023 (#direct_invoice, completely unguarded), 9711 (split payment, completely unguarded). The latter two had no flag check at all and so crashed for ANY waiter. VERIFIED on the production session shape (designation=Waiter, is_waiter=No, hidden INPUT, waiter_app_status renders 'No'), user's exact steps - Cup Yogurt, total 3000.00, Place Order: v3.6 -&gt; TypeError reading 'data', 0 order requests; v3.7 -&gt; no error, POST Sale/add_kitchen_sale_by_ajax fires. Admin regression same build: no crash, waiter dropdown still opens (select2-container--open=2), so behaviour unchanged where a real select2 exists. DEPLOY: commit 48936b4e - pos_script_v7.3.js + main_screen.php carrying ?v=3.6-&gt;3.7 in the SAME commit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Register</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Admin Register Management - force-close a register on someone else's behalf</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Done - verified</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Admin/Manager screen listing every open register across accessible outlets, with a force-close that reconciles a register abandoned by whoever opened it. DESIGN DECISIONS (user-confirmed before build): (1) the admin must TYPE the actually-counted cash, shown beside the system-computed figure - never a one-click accept, or the close stops catching discrepancies, which is its whole purpose; (2) calculation window is the register's own opening time to the moment of the click, same as a normal close, no backdating; (3) accountability is recorded - who force-closed, when, whose register, and why; (4) the discrepancy is stored in DEDICATED COLUMNS (system_closing_balance, force_closed_by, force_close_reason) rather than only as audit-log prose, given what it protects. REUSE: the arithmetic lives in Sale::closeRegister() plus six Sale_model methods that read counter_id/outlet_id from the SESSION, so they cannot compute for someone else's register. Added seven parameterised *ForRegister() twins taking counter_id/outlet_id explicitly, SQL byte-identical to the originals; the originals were left untouched so the normal per-user close is unaffected. Race guarded by WHERE id=? AND register_status=1 with an affected_rows() check. THREE PRE-EXISTING BUGS FOUND BY ACTUALLY RUNNING IT, not by reading it: (a) getAccessibleOutletIds() leaked an unterminated CI3 query-builder chain into its next query, so ANY non-Admin caller hit "Column 'id' in field list is ambiguous" - fixed with reset_query(); (b) the Register controller never loaded Sale_model; (c) the new JS called toastr, which userHome.php does not load (only the POS layout does) - switched to swal after confirming the bundled library is really SweetAlert v1. MENU/VERIFICATION LESSON - THE EXPENSIVE PART: the user could not see the menu item for several rounds while I reported it verified. Both claims were true and both missed each other: the &lt;li&gt; really was in userHome.php, and my DOM proof was real - but it was run against the SCRATCH database with the migration applied, while the user was looking at PRODUCTION, where it was not. Menu items are filtered client-side by user_home_buttom.js against window.menu_objects, built from the session's function_access, which is snapshotted from tbl_access AT LOGIN - so with no tbl_access row the entry is stripped from the DOM for everyone including Admin, and re-login cannot help because the row it reads does not exist. The same missing row also emptied the role-permission checkbox, which the user reported as a second symptom; it was the same cause. LESSON: 'verified' must name the database it was verified against, and a component proof on scratch is not evidence about production. RESOLUTION: migration applied to live 2026-09-04 after a mysqldump of tbl_register/tbl_access/tbl_role_access (db/backups/, gitignored) - tbl_access id 381, granted to Admin+Manager, 3 nullable columns added, register rows 24 before and after. Menu placement then changed twice on request: out of the Report submenu to a standalone top-level item above Report, plus an Admin-only header button beside the light/dark switch. The header button is gated by a DIRECT role check rather than data-access/menu_assign_class, matching the existing todays_summary button, so it does not depend on tbl_access or on re-login; the controller still gates the route via checkAccess(). Verified with the permission row deleted to mirror production exactly: button visible, sidebar entry correctly still hidden. User confirmed end-to-end on their own live account: 'tested ok'. DEPLOY: commits 84a0f165 (feature) and ef75e0ec (menu placement).</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Redesign</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>POS category rail - 3D depth, larger wrapping labels (client visual request)</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Done - verified</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Client compared the live rail against the originally approved reference and asked for more 3D depth and BIGGER buttons - explicitly taller, not wider. Delivered in two rounds. ROUND 1 offered two variants behind a ?rxcat= switch so the client could compare on their own till against the reference image, since this is a subjective visual call: v1 raised/42px, v2 bold/53px. Measured in-browser at 1440x900 against the rail's real calc(100vh - 120px) box: width stayed 130px in both (the brief's hard constraint - .list-of-item is a fixed column, so nothing outside the rail moves), heights 30 -&gt; 42 -&gt; 53, categories visible before scrolling 22 -&gt; 16 -&gt; 13 of 23. A third variant that wrapped labels was built and CUT: it overshot to 77px because the longest names take three lines at 130px, leaving only 9 visible. ROUND 2 - client picked v2, and separately lifted the single-line constraint: wrapping is preferred over truncation. So labels went 15px/600 -&gt; 17px/800 with white-space:normal, the ellipsis and nowrap from style2.css:399 overridden, and NO line-clamp, so a button grows to fit its name rather than the name being cut to fit the button. Height became a 56px FLOOR rather than a fixed value. FONT TRAP CAUGHT: the app's base Montserrat @import (style.css:2) loads 300-700 only, so the requested weight 800 would have rendered as a synthesised fake-bold. Added an explicit 800 link in main_screen.php - same family and host, so it adds a weight rather than another typeface. DEPTH RECIPE: three parts, not one shadow - a solid inset bottom edge reading as the button's thickness, an outer cast shadow lifting it off the rail, and an inset top highlight so the face looks lit from above; :active collapses the edge by its own thickness so the press reads as physical. The sheen is background-IMAGE, which layers over the per-category background-color set by the data-cix rules without restating eight colours per rule. TRADE ACCEPTED KNOWINGLY: taller buttons mean fewer categories reachable without scrolling. This supersedes the deliberate height decision in theme section 16; that comment is now marked superseded rather than deleted, so the original reasoning is not lost. Client confirmed the trade twice. Round 1 measured 13 of 23; round 2's larger text pushes it to roughly 11-12, which was flagged to the client as a CHANGE from the number they signed off rather than reported as still 13 - the final figure is calculated, not measured, because browser navigation to the local server was blocked during round 2. Side benefit worth keeping: at a 56px floor every button clears the 44px minimum normally recommended for a touch target; the old 30px rail did not, so this is a handling improvement and not only cosmetic. PROCESS NOTE: a sed one-liner used for the CSS cache-buster silently converted userHome.php from CRLF to LF, turning a 1-line change into a 2344-line diff. Caught with git diff --ignore-cr-at-eol before committing, reverted, and re-applied with an editor that preserves the file's bytes. Worth remembering on this repo - its files are not uniformly LF. PREVIEW ARTIFACT: claude.ai/code/artifact/22a01b29-7703-4814-b04d-677f2f8ae727 - renders the before/after at true 130px size from the same CSS values and typeface as the committed theme. DEPLOY: commit f76a2106, theme section 22, cache-buster v7.7.1.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
doc: sync the Task Tracker with what is actually built
The tracker had drifted. One row was wrong and five pieces of delivered work
had no row at all, which makes it an unreliable thing to plan from.

Corrected: the Hotel Operations Add-on still read "Not started". It is built
and live - three migrations, its own controller and views, two documents.

Added, all previously unrecorded: the POS Food/Drinks/Search work ("Part B",
whose roadmap note still claims "local only, not on live"), the table-first
ordering flow, the Waiter's Register Report, the S7 two-way merge, and the
local server optimisation batch.

Two of the new rows are deliberately marked NOT YET DEPLOYED and one reads
"Built - never run against live data", because a tracker that says Done for
something no client has received is worse than no tracker.

Register force-close was already recorded correctly at r79 (Done - verified);
no change was needed there.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/doc/Rexlio_POS_Task_Tracker.xlsx
+++ b/doc/Rexlio_POS_Task_Tracker.xlsx
@@ -611,7 +611,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E80"/>
+  <dimension ref="A1:E85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2065,7 +2065,7 @@
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done - built and live</t>
         </is>
       </c>
       <c r="D54" s="6" t="inlineStr">
@@ -2075,7 +2075,7 @@
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
-          <t>Scope finalized: Housekeeping + Front Desk basics only, isolated/toggleable add-on, new tables only. Reservations and Guest Folio explicitly excluded for now. Worth revisiting whether integration with the existing iLodge hotel product is better than duplicating hotel logic here.</t>
+          <t>BUILT. Housekeeping + Front Desk delivered as an isolated add-on behind the module switch. Schema migration 2026-09-16_02, stay value 2026-09-17_01, reports permission 2026-09-17_02. Controller application/controllers/Hotel.php, views application/views/hotel. Documented in doc/HOTEL_OPERATIONS_GUIDE.md and doc/GO_LIVE_HOTEL_2026-09-16.md. Reservations and Guest Folio remain out of scope.</t>
         </is>
       </c>
     </row>
@@ -2778,6 +2778,141 @@
       <c r="E80" t="inlineStr">
         <is>
           <t>Client compared the live rail against the originally approved reference and asked for more 3D depth and BIGGER buttons - explicitly taller, not wider. Delivered in two rounds. ROUND 1 offered two variants behind a ?rxcat= switch so the client could compare on their own till against the reference image, since this is a subjective visual call: v1 raised/42px, v2 bold/53px. Measured in-browser at 1440x900 against the rail's real calc(100vh - 120px) box: width stayed 130px in both (the brief's hard constraint - .list-of-item is a fixed column, so nothing outside the rail moves), heights 30 -&gt; 42 -&gt; 53, categories visible before scrolling 22 -&gt; 16 -&gt; 13 of 23. A third variant that wrapped labels was built and CUT: it overshot to 77px because the longest names take three lines at 130px, leaving only 9 visible. ROUND 2 - client picked v2, and separately lifted the single-line constraint: wrapping is preferred over truncation. So labels went 15px/600 -&gt; 17px/800 with white-space:normal, the ellipsis and nowrap from style2.css:399 overridden, and NO line-clamp, so a button grows to fit its name rather than the name being cut to fit the button. Height became a 56px FLOOR rather than a fixed value. FONT TRAP CAUGHT: the app's base Montserrat @import (style.css:2) loads 300-700 only, so the requested weight 800 would have rendered as a synthesised fake-bold. Added an explicit 800 link in main_screen.php - same family and host, so it adds a weight rather than another typeface. DEPTH RECIPE: three parts, not one shadow - a solid inset bottom edge reading as the button's thickness, an outer cast shadow lifting it off the rail, and an inset top highlight so the face looks lit from above; :active collapses the edge by its own thickness so the press reads as physical. The sheen is background-IMAGE, which layers over the per-category background-color set by the data-cix rules without restating eight colours per rule. TRADE ACCEPTED KNOWINGLY: taller buttons mean fewer categories reachable without scrolling. This supersedes the deliberate height decision in theme section 16; that comment is now marked superseded rather than deleted, so the original reasoning is not lost. Client confirmed the trade twice. Round 1 measured 13 of 23; round 2's larger text pushes it to roughly 11-12, which was flagged to the client as a CHANGE from the number they signed off rather than reported as still 13 - the final figure is calculated, not measured, because browser navigation to the local server was blocked during round 2. Side benefit worth keeping: at a 56px floor every button clears the 44px minimum normally recommended for a touch target; the old 30px rail did not, so this is a handling improvement and not only cosmetic. PROCESS NOTE: a sed one-liner used for the CSS cache-buster silently converted userHome.php from CRLF to LF, turning a 1-line change into a 2344-line diff. Caught with git diff --ignore-cr-at-eol before committing, reverted, and re-applied with an editor that preserves the file's bytes. Worth remembering on this repo - its files are not uniformly LF. PREVIEW ARTIFACT: claude.ai/code/artifact/22a01b29-7703-4814-b04d-677f2f8ae727 - renders the before/after at true 130px size from the same CSS values and typeface as the committed theme. DEPLOY: commit f76a2106, theme section 22, cache-buster v7.7.1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Phase B</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>POS Sale screen - Food / Drinks toggle, Search button, search clears ("Part B")</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Done - built and live</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Delivered 2026-09-15. The roadmap (line 297) still carries the note "Local only; not on live", which is stale - both clients are well past that commit. 18/18 regression suite, referenced throughout doc/HOTEL_ADDON_PLAN.md as the Part B baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Phase B</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Table-first ordering flow</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Done - built and live</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Migration 2026-09-15_04_table-first-flow.sql. Plan and decisions in doc/TABLE_FIRST_FLOW_PLAN.md. Tables panel regression 55/22/28/16. Was never given a tracker row.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Waiter's Register Report - one waiter's own takings for one register session</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Done - NOT YET DEPLOYED</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Built 2026-09-25. Filtered view of the Register Report plus the waiter's voided/cancelled orders from tbl_audit_logs, a completed-orders list and a print button. Reached from the Report menu and the waiter panel. Needs migration 2026-09-25_01_waiter-register-report.sql on each client. Commits 30e17af5, 54ca0cfd, 38e0a894, 6383ab7b. Waiters must log out and back in to pick up the permission.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Sync</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>S7 - two-way merge between the local server and the online copy</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Built - never run against live data</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Deployment Manager gained a merge engine: orders, their edits and voids, running orders to the kitchen screen, customers matched on phone, catalogue push. Insert-only; only the side that created an order may change it; nothing is ever deleted. 144 checks pass on practice databases and the readiness check passes against the real Rockbell host. THE FIRST REAL MERGE HAS NOT BEEN RUN. Do it on a quiet morning, watched, after confirming the live backup.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Perf</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Local server optimisation - no internet fetches, no animation delay</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Done - NOT YET DEPLOYED</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Core pages were fetching fonts from fonts.googleapis.com (measured 1.43s, render-blocking, and a stall at a venue with no internet) - now served locally. Page preloader wasted a full second after load; jQuery.fx off, animate.css forced to 0s. Login measured 0.82s end to end, 12 requests, none external. Commit b43816a2. Machine config (php.ini OPcache, my.ini) does NOT deploy - see Technical Guide v2.8 "Production Server Setup Checklist".</t>
         </is>
       </c>
     </row>

</xml_diff>